<commit_message>
Framework - Added Skip test cases flag - 02 April 2026
</commit_message>
<xml_diff>
--- a/SeleniumJavaFramework/TestData/TestData.xlsx
+++ b/SeleniumJavaFramework/TestData/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tales\git\SeleniumFramework\SeleniumJavaFramework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FD2940-1403-42F1-83CE-7D3FB3629317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E71423-4F75-4240-A837-D40F936EC4C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FrenchMappings" sheetId="38" state="hidden" r:id="rId1"/>
@@ -26,7 +26,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FrenchMappings!$A$1:$D$372</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">FrenchMappingsOld!$A$1:$D$140</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TestCases!$A$1:$U$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TestCases!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">testSupportTypeForms!$E$1:$E$34</definedName>
     <definedName name="Browsers_Devices">Dropdowns!$C$2:$C$12</definedName>
     <definedName name="Product_Services">Dropdowns!$A$2:$A$6</definedName>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2572" uniqueCount="977">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2539" uniqueCount="962">
   <si>
     <t>Module</t>
   </si>
@@ -2398,18 +2398,6 @@
     <t>12-57854-53001</t>
   </si>
   <si>
-    <t>testAutoPayEnrollment</t>
-  </si>
-  <si>
-    <t>testEnrollmentElegiblityForAutopay</t>
-  </si>
-  <si>
-    <t>testDefaultContentForAutopay</t>
-  </si>
-  <si>
-    <t>Release</t>
-  </si>
-  <si>
     <t>logged in State</t>
   </si>
   <si>
@@ -2518,9 +2506,6 @@
     <t>redirectionFrom</t>
   </si>
   <si>
-    <t>testRequestFormSubmission</t>
-  </si>
-  <si>
     <t>1111130169</t>
   </si>
   <si>
@@ -2962,9 +2947,6 @@
     <t>https://wmqa2.wm.com/ca/fr/myhome</t>
   </si>
   <si>
-    <t>AutoPay</t>
-  </si>
-  <si>
     <t>autotester@testmail.com</t>
   </si>
   <si>
@@ -2992,9 +2974,6 @@
     <t>isLAAddress</t>
   </si>
   <si>
-    <t>S8</t>
-  </si>
-  <si>
     <t>94601</t>
   </si>
   <si>
@@ -3016,39 +2995,6 @@
     <t>state</t>
   </si>
   <si>
-    <t>IE11</t>
-  </si>
-  <si>
-    <t>S7</t>
-  </si>
-  <si>
-    <t>S6</t>
-  </si>
-  <si>
-    <t>iPhone7</t>
-  </si>
-  <si>
-    <t>iPhone7+</t>
-  </si>
-  <si>
-    <t>iPhone X</t>
-  </si>
-  <si>
-    <t>iPhone X Max</t>
-  </si>
-  <si>
-    <t>iPad Pro</t>
-  </si>
-  <si>
-    <t>iPad Mini</t>
-  </si>
-  <si>
-    <t>Phase 6</t>
-  </si>
-  <si>
-    <t>Merge</t>
-  </si>
-  <si>
     <t>DBICMS-2477/DBICMS-1653/Verify the submission of the extra pickup form.</t>
   </si>
   <si>
@@ -3095,6 +3041,15 @@
   </si>
   <si>
     <t>https://oshoworld.com/</t>
+  </si>
+  <si>
+    <t>testBrowserOpenURL</t>
+  </si>
+  <si>
+    <t>Practice</t>
+  </si>
+  <si>
+    <t>testDropDownElement</t>
   </si>
 </sst>
 </file>
@@ -3331,14 +3286,14 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>5869388</xdr:colOff>
-          <xdr:row>310</xdr:row>
-          <xdr:rowOff>7620</xdr:rowOff>
+          <xdr:row>298</xdr:row>
+          <xdr:rowOff>184205</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>265375</xdr:colOff>
-          <xdr:row>311</xdr:row>
-          <xdr:rowOff>104030</xdr:rowOff>
+          <xdr:row>300</xdr:row>
+          <xdr:rowOff>95084</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -4233,7 +4188,7 @@
         <v>347</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>900</v>
+        <v>895</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="28.8">
@@ -4367,10 +4322,10 @@
         <v>173</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -6202,10 +6157,10 @@
         <v>162</v>
       </c>
       <c r="B182" s="11" t="s">
-        <v>935</v>
+        <v>929</v>
       </c>
       <c r="C182" s="11" t="s">
-        <v>935</v>
+        <v>929</v>
       </c>
       <c r="D182" s="11">
         <f t="shared" si="3"/>
@@ -7042,10 +6997,10 @@
         <v>387</v>
       </c>
       <c r="B238" s="16" t="s">
-        <v>903</v>
+        <v>898</v>
       </c>
       <c r="C238" s="16" t="s">
-        <v>904</v>
+        <v>899</v>
       </c>
       <c r="D238" s="11">
         <f t="shared" si="3"/>
@@ -7300,7 +7255,7 @@
         <v>582</v>
       </c>
       <c r="C255" s="11" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="D255" s="11">
         <f t="shared" si="4"/>
@@ -7552,10 +7507,10 @@
         <v>570</v>
       </c>
       <c r="B272" s="11" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="C272" s="11" t="s">
-        <v>907</v>
+        <v>902</v>
       </c>
       <c r="D272" s="11">
         <f t="shared" si="4"/>
@@ -8110,7 +8065,7 @@
         <v>665</v>
       </c>
       <c r="C309" s="11" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="D309" s="11">
         <f t="shared" si="5"/>
@@ -8122,10 +8077,10 @@
         <v>17</v>
       </c>
       <c r="B310" s="11" t="s">
-        <v>909</v>
+        <v>904</v>
       </c>
       <c r="C310" s="11" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="D310" s="11">
         <f t="shared" si="5"/>
@@ -8137,10 +8092,10 @@
         <v>17</v>
       </c>
       <c r="B311" s="11" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="C311" s="11" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="D311" s="11">
         <f t="shared" si="5"/>
@@ -8272,10 +8227,10 @@
         <v>17</v>
       </c>
       <c r="B320" s="11" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
       <c r="C320" s="11" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="D320" s="11" t="e">
         <f t="shared" si="5"/>
@@ -9112,10 +9067,10 @@
         <v>155</v>
       </c>
       <c r="B376" s="11" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="C376" s="11" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="D376" s="11">
         <f t="shared" si="6"/>
@@ -9127,10 +9082,10 @@
         <v>570</v>
       </c>
       <c r="B377" s="11" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
       <c r="C377" s="11" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
       <c r="D377" s="11">
         <f t="shared" si="6"/>
@@ -9142,10 +9097,10 @@
         <v>582</v>
       </c>
       <c r="B378" s="11" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
       <c r="C378" s="11" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="D378" s="11">
         <f t="shared" si="6"/>
@@ -9157,10 +9112,10 @@
         <v>396</v>
       </c>
       <c r="B379" s="11" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="C379" s="11" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="D379" s="11">
         <f t="shared" si="6"/>
@@ -9172,10 +9127,10 @@
         <v>396</v>
       </c>
       <c r="B380" s="11" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="C380" s="11" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
       <c r="D380" s="11">
         <v>1</v>
@@ -9186,10 +9141,10 @@
         <v>396</v>
       </c>
       <c r="B381" s="11" t="s">
-        <v>925</v>
+        <v>920</v>
       </c>
       <c r="C381" s="11" t="s">
-        <v>926</v>
+        <v>921</v>
       </c>
     </row>
     <row r="382" spans="1:4">
@@ -9197,21 +9152,21 @@
         <v>396</v>
       </c>
       <c r="B382" s="11" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
       <c r="C382" s="11" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
     </row>
     <row r="383" spans="1:4">
       <c r="A383" s="11" t="s">
-        <v>929</v>
+        <v>924</v>
       </c>
       <c r="B383" t="s">
-        <v>930</v>
+        <v>925</v>
       </c>
       <c r="C383" t="s">
-        <v>931</v>
+        <v>926</v>
       </c>
     </row>
     <row r="384" spans="1:4">
@@ -9222,7 +9177,7 @@
         <v>665</v>
       </c>
       <c r="C384" s="11" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
     </row>
     <row r="385" spans="1:3">
@@ -9230,10 +9185,10 @@
         <v>396</v>
       </c>
       <c r="B385" s="11" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="C385" s="11" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
     </row>
     <row r="386" spans="1:3">
@@ -9241,10 +9196,10 @@
         <v>396</v>
       </c>
       <c r="B386" s="11" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="C386" s="11" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
     </row>
   </sheetData>
@@ -9268,14 +9223,14 @@
               <from>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>310</xdr:row>
-                <xdr:rowOff>7620</xdr:rowOff>
+                <xdr:row>299</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>266700</xdr:colOff>
-                <xdr:row>311</xdr:row>
-                <xdr:rowOff>106680</xdr:rowOff>
+                <xdr:row>300</xdr:row>
+                <xdr:rowOff>91440</xdr:rowOff>
               </to>
             </anchor>
           </controlPr>
@@ -11369,19 +11324,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BB88851-103F-462A-BEFE-119AAEDB1A91}">
   <sheetPr codeName="Sheet33"/>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="16.44140625" defaultRowHeight="18.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.88671875" style="22" customWidth="1"/>
-    <col min="2" max="2" width="46.88671875" style="22" customWidth="1"/>
+    <col min="2" max="2" width="22.88671875" style="22" customWidth="1"/>
     <col min="3" max="3" width="14.5546875" style="29" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="16.44140625" style="29"/>
-    <col min="7" max="7" width="13.5546875" style="29" customWidth="1"/>
-    <col min="8" max="21" width="10.6640625" style="29" customWidth="1"/>
-    <col min="22" max="16384" width="16.44140625" style="29"/>
+    <col min="4" max="16384" width="16.44140625" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="18.75" customHeight="1">
+    <row r="1" spans="1:6" ht="18.75" customHeight="1">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -11400,58 +11352,13 @@
       <c r="F1" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="21" t="s">
-        <v>747</v>
-      </c>
-      <c r="H1" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="21" t="s">
-        <v>950</v>
-      </c>
-      <c r="J1" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="K1" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="L1" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="M1" s="21" t="s">
-        <v>942</v>
-      </c>
-      <c r="N1" s="21" t="s">
-        <v>951</v>
-      </c>
-      <c r="O1" s="21" t="s">
-        <v>952</v>
-      </c>
-      <c r="P1" s="21" t="s">
-        <v>953</v>
-      </c>
-      <c r="Q1" s="21" t="s">
-        <v>954</v>
-      </c>
-      <c r="R1" s="21" t="s">
-        <v>955</v>
-      </c>
-      <c r="S1" s="21" t="s">
-        <v>956</v>
-      </c>
-      <c r="T1" s="21" t="s">
-        <v>957</v>
-      </c>
-      <c r="U1" s="21" t="s">
-        <v>958</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" ht="18.75" customHeight="1">
+    </row>
+    <row r="2" spans="1:6" ht="18.75" customHeight="1">
       <c r="A2" s="30" t="s">
-        <v>932</v>
+        <v>960</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>744</v>
+        <v>959</v>
       </c>
       <c r="C2" s="29" t="s">
         <v>9</v>
@@ -11462,96 +11369,34 @@
       <c r="E2" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="29" t="s">
-        <v>959</v>
-      </c>
-      <c r="H2" s="29" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A3" s="22" t="s">
-        <v>932</v>
+    </row>
+    <row r="3" spans="1:6" ht="18.75" customHeight="1">
+      <c r="A3" s="30" t="s">
+        <v>960</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>745</v>
+        <v>961</v>
       </c>
       <c r="C3" s="29" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>114</v>
-      </c>
-      <c r="G3" s="29" t="s">
-        <v>959</v>
-      </c>
-      <c r="H3" s="29" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A4" s="22" t="s">
-        <v>932</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>746</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="29" t="s">
-        <v>114</v>
-      </c>
-      <c r="G4" s="29" t="s">
-        <v>959</v>
-      </c>
-      <c r="H4" s="29" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A5" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>784</v>
-      </c>
-      <c r="C5" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="29" t="s">
-        <v>114</v>
-      </c>
-      <c r="G5" s="29" t="s">
-        <v>960</v>
-      </c>
-      <c r="H5" s="29" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U5" xr:uid="{58BB8307-DA66-45F3-826C-C44C0A3BE5B2}"/>
+  <autoFilter ref="A1:F2" xr:uid="{58BB8307-DA66-45F3-826C-C44C0A3BE5B2}"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E5" xr:uid="{DD5ACA89-92FD-4A3F-8807-B6CAEA85C9AF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3" xr:uid="{DD5ACA89-92FD-4A3F-8807-B6CAEA85C9AF}">
       <formula1>INDIRECT("Browsers_Devices")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D5" xr:uid="{5D9E317B-E2F4-470E-A05D-363E1676010C}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3" xr:uid="{5D9E317B-E2F4-470E-A05D-363E1676010C}">
       <formula1>INDIRECT("TEST_Category")</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="B2" location="testAutoPayEnrollment!A2" display="testAutoPayEnrollment" xr:uid="{21AF9365-3455-46BE-AF64-F1BC1C2A04D7}"/>
-    <hyperlink ref="B5" location="testRequestFormSubmission!A2" display="testRequestFormSubmission" xr:uid="{6AA625B5-C86C-4A44-B096-5AA52668B846}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -11577,40 +11422,40 @@
         <v>378</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>972</v>
+        <v>954</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="10" t="s">
-        <v>973</v>
+        <v>955</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>136</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>974</v>
+        <v>956</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="28.8">
       <c r="A3" s="10" t="s">
-        <v>973</v>
+        <v>955</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>136</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>975</v>
+        <v>957</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="10" t="s">
-        <v>973</v>
+        <v>955</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>136</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>976</v>
+        <v>958</v>
       </c>
     </row>
   </sheetData>
@@ -11662,108 +11507,108 @@
         <v>378</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="E1" s="17" t="s">
         <v>379</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>899</v>
+        <v>894</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>898</v>
+        <v>893</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>804</v>
+        <v>799</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
       <c r="J1" s="17" t="s">
         <v>278</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="L1" s="17" t="s">
         <v>405</v>
       </c>
       <c r="M1" s="17" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="N1" s="17" t="s">
         <v>393</v>
       </c>
       <c r="O1" s="17" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="P1" s="17" t="s">
-        <v>949</v>
+        <v>942</v>
       </c>
       <c r="Q1" s="17" t="s">
         <v>26</v>
       </c>
       <c r="R1" s="17" t="s">
-        <v>941</v>
+        <v>935</v>
       </c>
       <c r="S1" s="17" t="s">
-        <v>940</v>
+        <v>934</v>
       </c>
       <c r="T1" s="17" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="U1" s="17" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="V1" s="17" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="W1" s="17" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="X1" s="17" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="Y1" s="17" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
     </row>
     <row r="2" spans="1:25" s="20" customFormat="1" ht="28.8">
       <c r="A2" s="20" t="s">
-        <v>948</v>
+        <v>941</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>861</v>
+        <v>856</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J2" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K2" s="23" t="s">
-        <v>859</v>
+        <v>854</v>
       </c>
       <c r="L2" s="7" t="s">
         <v>743</v>
@@ -11779,15 +11624,15 @@
         <v>28</v>
       </c>
       <c r="Q2" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R2" s="24"/>
       <c r="S2" s="24"/>
       <c r="T2" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V2" s="5" t="s">
         <v>402</v>
@@ -11802,40 +11647,40 @@
     </row>
     <row r="3" spans="1:25" s="20" customFormat="1" ht="28.8">
       <c r="A3" s="20" t="s">
-        <v>947</v>
+        <v>940</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D3" s="24" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E3" s="24" t="s">
         <v>35</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>946</v>
+        <v>939</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K3" s="23" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>945</v>
+        <v>938</v>
       </c>
       <c r="M3" s="5"/>
       <c r="N3" s="5" t="s">
@@ -11848,15 +11693,15 @@
         <v>28</v>
       </c>
       <c r="Q3" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R3" s="24"/>
       <c r="S3" s="24"/>
       <c r="T3" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V3" s="5" t="s">
         <v>402</v>
@@ -11870,40 +11715,40 @@
     </row>
     <row r="4" spans="1:25" ht="28.8">
       <c r="A4" s="5" t="s">
-        <v>966</v>
+        <v>948</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>946</v>
+        <v>939</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K4" s="23" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>945</v>
+        <v>938</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>402</v>
@@ -11915,17 +11760,17 @@
         <v>28</v>
       </c>
       <c r="Q4" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R4" s="24"/>
       <c r="S4" s="24" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V4" s="5" t="s">
         <v>402</v>
@@ -11939,40 +11784,40 @@
     </row>
     <row r="5" spans="1:25" ht="28.8">
       <c r="A5" s="5" t="s">
-        <v>965</v>
+        <v>947</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>946</v>
+        <v>939</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K5" s="23" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>945</v>
+        <v>938</v>
       </c>
       <c r="N5" s="5" t="s">
         <v>402</v>
@@ -11984,15 +11829,15 @@
         <v>28</v>
       </c>
       <c r="Q5" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R5" s="24"/>
       <c r="S5" s="24"/>
       <c r="T5" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V5" s="5" t="s">
         <v>402</v>
@@ -12006,43 +11851,43 @@
     </row>
     <row r="6" spans="1:25" ht="28.8">
       <c r="A6" s="5" t="s">
-        <v>944</v>
+        <v>937</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J6" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K6" s="23" t="s">
-        <v>868</v>
+        <v>863</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>867</v>
+        <v>862</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>402</v>
@@ -12054,15 +11899,15 @@
         <v>28</v>
       </c>
       <c r="Q6" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R6" s="24"/>
       <c r="S6" s="24"/>
       <c r="T6" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V6" s="5" t="s">
         <v>402</v>
@@ -12076,40 +11921,40 @@
     </row>
     <row r="7" spans="1:25" ht="29.25" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>964</v>
+        <v>946</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D7" s="24" t="s">
+        <v>881</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>891</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>886</v>
       </c>
-      <c r="E7" s="24" t="s">
-        <v>896</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>891</v>
-      </c>
       <c r="G7" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J7" s="27" t="s">
+        <v>927</v>
+      </c>
+      <c r="K7" s="23" t="s">
+        <v>884</v>
+      </c>
+      <c r="L7" s="7" t="s">
         <v>933</v>
-      </c>
-      <c r="K7" s="23" t="s">
-        <v>889</v>
-      </c>
-      <c r="L7" s="7" t="s">
-        <v>939</v>
       </c>
       <c r="N7" s="5" t="s">
         <v>402</v>
@@ -12121,17 +11966,17 @@
         <v>28</v>
       </c>
       <c r="Q7" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R7" s="24"/>
       <c r="S7" s="24" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="T7" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>402</v>
@@ -12145,40 +11990,40 @@
     </row>
     <row r="8" spans="1:25" s="20" customFormat="1" ht="28.8">
       <c r="A8" s="20" t="s">
-        <v>963</v>
+        <v>945</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>861</v>
+        <v>856</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J8" s="27" t="s">
+        <v>927</v>
+      </c>
+      <c r="K8" s="23" t="s">
+        <v>854</v>
+      </c>
+      <c r="L8" s="7" t="s">
         <v>933</v>
-      </c>
-      <c r="K8" s="23" t="s">
-        <v>859</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>939</v>
       </c>
       <c r="M8" s="5"/>
       <c r="N8" s="5" t="s">
@@ -12191,17 +12036,17 @@
         <v>28</v>
       </c>
       <c r="Q8" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R8" s="24"/>
       <c r="S8" s="24" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="T8" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V8" s="5" t="s">
         <v>402</v>
@@ -12216,16 +12061,16 @@
     </row>
     <row r="9" spans="1:25" ht="28.8">
       <c r="A9" s="5" t="s">
-        <v>808</v>
+        <v>803</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>35</v>
@@ -12234,25 +12079,25 @@
         <v>303</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J9" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K9" s="23" t="s">
-        <v>806</v>
+        <v>801</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N9" s="5" t="s">
         <v>402</v>
@@ -12264,14 +12109,14 @@
         <v>28</v>
       </c>
       <c r="Q9" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R9" s="24"/>
       <c r="T9" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V9" s="5" t="s">
         <v>402</v>
@@ -12285,43 +12130,43 @@
     </row>
     <row r="10" spans="1:25" ht="28.8">
       <c r="A10" s="5" t="s">
-        <v>852</v>
+        <v>847</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>851</v>
+        <v>846</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>40</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>850</v>
+        <v>845</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J10" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K10" s="23" t="s">
-        <v>849</v>
+        <v>844</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>848</v>
+        <v>843</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N10" s="5" t="s">
         <v>402</v>
@@ -12333,15 +12178,15 @@
         <v>28</v>
       </c>
       <c r="Q10" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R10" s="24"/>
       <c r="S10" s="24"/>
       <c r="T10" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V10" s="5" t="s">
         <v>402</v>
@@ -12355,43 +12200,43 @@
     </row>
     <row r="11" spans="1:25" ht="28.8">
       <c r="A11" s="5" t="s">
-        <v>866</v>
+        <v>861</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F11" s="5" t="s">
+        <v>860</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>865</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>870</v>
-      </c>
       <c r="H11" s="5" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J11" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K11" s="23" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>862</v>
+        <v>857</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N11" s="5" t="s">
         <v>402</v>
@@ -12403,15 +12248,15 @@
         <v>28</v>
       </c>
       <c r="Q11" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R11" s="24"/>
       <c r="S11" s="24"/>
       <c r="T11" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V11" s="5" t="s">
         <v>402</v>
@@ -12425,43 +12270,43 @@
     </row>
     <row r="12" spans="1:25" ht="28.8">
       <c r="A12" s="5" t="s">
-        <v>847</v>
+        <v>842</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>846</v>
+        <v>841</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>845</v>
+        <v>840</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J12" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K12" s="23" t="s">
-        <v>844</v>
+        <v>839</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>843</v>
+        <v>838</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N12" s="5" t="s">
         <v>402</v>
@@ -12473,15 +12318,15 @@
         <v>28</v>
       </c>
       <c r="Q12" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R12" s="24"/>
       <c r="S12" s="24"/>
       <c r="T12" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U12" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V12" s="5" t="s">
         <v>402</v>
@@ -12495,43 +12340,43 @@
     </row>
     <row r="13" spans="1:25" ht="28.8">
       <c r="A13" s="5" t="s">
-        <v>842</v>
+        <v>837</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>841</v>
+        <v>836</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>840</v>
+        <v>835</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J13" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K13" s="23" t="s">
-        <v>839</v>
+        <v>834</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>838</v>
+        <v>833</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N13" s="5" t="s">
         <v>402</v>
@@ -12543,15 +12388,15 @@
         <v>28</v>
       </c>
       <c r="Q13" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R13" s="24"/>
       <c r="S13" s="24"/>
       <c r="T13" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U13" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V13" s="5" t="s">
         <v>402</v>
@@ -12565,43 +12410,43 @@
     </row>
     <row r="14" spans="1:25" ht="28.8">
       <c r="A14" s="5" t="s">
-        <v>837</v>
+        <v>832</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>836</v>
+        <v>831</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>835</v>
+        <v>830</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J14" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K14" s="23" t="s">
-        <v>834</v>
+        <v>829</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>833</v>
+        <v>828</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N14" s="5" t="s">
         <v>402</v>
@@ -12613,15 +12458,15 @@
         <v>28</v>
       </c>
       <c r="Q14" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R14" s="24"/>
       <c r="S14" s="24"/>
       <c r="T14" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V14" s="5" t="s">
         <v>402</v>
@@ -12635,37 +12480,37 @@
     </row>
     <row r="15" spans="1:25" s="24" customFormat="1" ht="36.75" customHeight="1">
       <c r="A15" s="28" t="s">
-        <v>897</v>
+        <v>892</v>
       </c>
       <c r="B15" s="24" t="s">
         <v>138</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H15" s="24" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="I15" s="24" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J15" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K15" s="26" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="L15" s="25"/>
       <c r="N15" s="24" t="s">
@@ -12678,13 +12523,13 @@
         <v>28</v>
       </c>
       <c r="Q15" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="T15" s="24" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U15" s="24" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V15" s="24" t="s">
         <v>402</v>
@@ -12698,40 +12543,40 @@
     </row>
     <row r="16" spans="1:25" ht="29.25" customHeight="1">
       <c r="A16" s="5" t="s">
-        <v>962</v>
+        <v>944</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D16" s="24" t="s">
+        <v>881</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>891</v>
+      </c>
+      <c r="F16" s="5" t="s">
         <v>886</v>
       </c>
-      <c r="E16" s="24" t="s">
-        <v>896</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>891</v>
-      </c>
       <c r="G16" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J16" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K16" s="23" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="N16" s="5" t="s">
         <v>402</v>
@@ -12743,15 +12588,15 @@
         <v>28</v>
       </c>
       <c r="Q16" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R16" s="24"/>
       <c r="S16" s="24"/>
       <c r="T16" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U16" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V16" s="5" t="s">
         <v>402</v>
@@ -12765,43 +12610,43 @@
     </row>
     <row r="17" spans="1:24" ht="28.8">
       <c r="A17" s="5" t="s">
-        <v>895</v>
+        <v>890</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J17" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K17" s="23" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>892</v>
+        <v>887</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N17" s="5" t="s">
         <v>402</v>
@@ -12813,15 +12658,15 @@
         <v>28</v>
       </c>
       <c r="Q17" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R17" s="24"/>
       <c r="S17" s="24"/>
       <c r="T17" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U17" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V17" s="5" t="s">
         <v>402</v>
@@ -12835,40 +12680,40 @@
     </row>
     <row r="18" spans="1:24" ht="29.25" customHeight="1">
       <c r="A18" s="5" t="s">
-        <v>938</v>
+        <v>932</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E18" s="24" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J18" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K18" s="23" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="N18" s="5" t="s">
         <v>402</v>
@@ -12880,15 +12725,15 @@
         <v>28</v>
       </c>
       <c r="Q18" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R18" s="24"/>
       <c r="S18" s="24"/>
       <c r="T18" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V18" s="5" t="s">
         <v>402</v>
@@ -12902,40 +12747,40 @@
     </row>
     <row r="19" spans="1:24" ht="28.8">
       <c r="A19" s="5" t="s">
-        <v>961</v>
+        <v>943</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>861</v>
+        <v>856</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J19" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K19" s="23" t="s">
-        <v>859</v>
+        <v>854</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="N19" s="5" t="s">
         <v>402</v>
@@ -12947,15 +12792,15 @@
         <v>28</v>
       </c>
       <c r="Q19" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R19" s="24"/>
       <c r="S19" s="24"/>
       <c r="T19" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V19" s="5" t="s">
         <v>402</v>
@@ -12969,43 +12814,43 @@
     </row>
     <row r="20" spans="1:24" ht="28.8">
       <c r="A20" s="5" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>855</v>
+        <v>850</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J20" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K20" s="23" t="s">
-        <v>854</v>
+        <v>849</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>853</v>
+        <v>848</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N20" s="5" t="s">
         <v>402</v>
@@ -13017,15 +12862,15 @@
         <v>28</v>
       </c>
       <c r="Q20" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R20" s="24"/>
       <c r="S20" s="24"/>
       <c r="T20" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V20" s="5" t="s">
         <v>402</v>
@@ -13039,43 +12884,43 @@
     </row>
     <row r="21" spans="1:24" ht="28.8">
       <c r="A21" s="5" t="s">
-        <v>872</v>
+        <v>867</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J21" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K21" s="23" t="s">
-        <v>868</v>
+        <v>863</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>867</v>
+        <v>862</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N21" s="5" t="s">
         <v>402</v>
@@ -13087,7 +12932,7 @@
         <v>28</v>
       </c>
       <c r="Q21" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R21" s="24"/>
       <c r="S21" s="24"/>
@@ -13097,28 +12942,28 @@
     </row>
     <row r="22" spans="1:24">
       <c r="A22" s="5" t="s">
-        <v>803</v>
+        <v>798</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="J22" s="27"/>
       <c r="K22" s="23"/>
@@ -13127,35 +12972,35 @@
         <v>28</v>
       </c>
       <c r="Q22" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R22" s="24"/>
       <c r="S22" s="24"/>
     </row>
     <row r="23" spans="1:24">
       <c r="A23" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="J23" s="27"/>
       <c r="K23" s="23"/>
@@ -13164,35 +13009,35 @@
         <v>28</v>
       </c>
       <c r="Q23" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R23" s="24"/>
       <c r="S23" s="24"/>
     </row>
     <row r="24" spans="1:24">
       <c r="A24" s="5" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="J24" s="27"/>
       <c r="K24" s="23"/>
@@ -13201,50 +13046,50 @@
         <v>28</v>
       </c>
       <c r="Q24" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R24" s="24"/>
       <c r="S24" s="24"/>
     </row>
     <row r="25" spans="1:24" ht="28.8">
       <c r="A25" s="5" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>380</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J25" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K25" s="23" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>867</v>
+        <v>862</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N25" s="5" t="s">
         <v>402</v>
@@ -13256,15 +13101,15 @@
         <v>28</v>
       </c>
       <c r="Q25" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R25" s="24"/>
       <c r="S25" s="24"/>
       <c r="T25" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U25" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V25" s="5" t="s">
         <v>402</v>
@@ -13278,28 +13123,28 @@
     </row>
     <row r="26" spans="1:24">
       <c r="A26" s="5" t="s">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="J26" s="27"/>
       <c r="K26" s="23"/>
@@ -13308,35 +13153,35 @@
         <v>28</v>
       </c>
       <c r="Q26" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R26" s="24"/>
       <c r="S26" s="24"/>
     </row>
     <row r="27" spans="1:24" ht="28.8">
       <c r="A27" s="5" t="s">
-        <v>879</v>
+        <v>874</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="J27" s="27"/>
       <c r="K27" s="23"/>
@@ -13345,50 +13190,50 @@
         <v>28</v>
       </c>
       <c r="Q27" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R27" s="24"/>
       <c r="S27" s="24"/>
     </row>
     <row r="28" spans="1:24" ht="28.8">
       <c r="A28" s="5" t="s">
-        <v>876</v>
+        <v>871</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>875</v>
+        <v>870</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>855</v>
+        <v>850</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J28" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K28" s="23" t="s">
-        <v>874</v>
+        <v>869</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>873</v>
+        <v>868</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N28" s="5" t="s">
         <v>402</v>
@@ -13400,15 +13245,15 @@
         <v>28</v>
       </c>
       <c r="Q28" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R28" s="24"/>
       <c r="S28" s="24"/>
       <c r="T28" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U28" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V28" s="5" t="s">
         <v>402</v>
@@ -13422,28 +13267,28 @@
     </row>
     <row r="29" spans="1:24" ht="28.8">
       <c r="A29" s="5" t="s">
-        <v>832</v>
+        <v>827</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>830</v>
+        <v>825</v>
       </c>
       <c r="J29" s="27"/>
       <c r="K29" s="23"/>
@@ -13452,50 +13297,50 @@
         <v>28</v>
       </c>
       <c r="Q29" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R29" s="24"/>
       <c r="S29" s="24"/>
     </row>
     <row r="30" spans="1:24" ht="28.8">
       <c r="A30" s="5" t="s">
-        <v>829</v>
+        <v>824</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>827</v>
+        <v>822</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J30" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K30" s="23" t="s">
-        <v>826</v>
+        <v>821</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>825</v>
+        <v>820</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N30" s="5" t="s">
         <v>402</v>
@@ -13507,15 +13352,15 @@
         <v>28</v>
       </c>
       <c r="Q30" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R30" s="24"/>
       <c r="S30" s="24"/>
       <c r="T30" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U30" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V30" s="5" t="s">
         <v>402</v>
@@ -13529,43 +13374,43 @@
     </row>
     <row r="31" spans="1:24" ht="28.8">
       <c r="A31" s="5" t="s">
-        <v>824</v>
+        <v>819</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>823</v>
+        <v>818</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>822</v>
+        <v>817</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J31" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K31" s="23" t="s">
-        <v>821</v>
+        <v>816</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>820</v>
+        <v>815</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N31" s="5" t="s">
         <v>402</v>
@@ -13577,15 +13422,15 @@
         <v>28</v>
       </c>
       <c r="Q31" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R31" s="24"/>
       <c r="S31" s="24"/>
       <c r="T31" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U31" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V31" s="5" t="s">
         <v>402</v>
@@ -13599,43 +13444,43 @@
     </row>
     <row r="32" spans="1:24" ht="28.8">
       <c r="A32" s="5" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E32" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>818</v>
+        <v>813</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>817</v>
+        <v>812</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="J32" s="27" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="K32" s="23" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="M32" s="5" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="N32" s="5" t="s">
         <v>402</v>
@@ -13647,15 +13492,15 @@
         <v>28</v>
       </c>
       <c r="Q32" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R32" s="24"/>
       <c r="S32" s="24"/>
       <c r="T32" s="5" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="U32" s="5" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="V32" s="5" t="s">
         <v>402</v>
@@ -13669,28 +13514,28 @@
     </row>
     <row r="33" spans="1:19">
       <c r="A33" s="5" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="J33" s="27"/>
       <c r="K33" s="23"/>
@@ -13699,35 +13544,35 @@
         <v>28</v>
       </c>
       <c r="Q33" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R33" s="24"/>
       <c r="S33" s="24"/>
     </row>
     <row r="34" spans="1:19" ht="28.8">
       <c r="A34" s="5" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>35</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="J34" s="27"/>
       <c r="K34" s="23"/>
@@ -13736,7 +13581,7 @@
         <v>28</v>
       </c>
       <c r="Q34" s="25" t="s">
-        <v>943</v>
+        <v>936</v>
       </c>
       <c r="R34" s="24"/>
       <c r="S34" s="24"/>
@@ -13831,7 +13676,7 @@
     </row>
     <row r="2" spans="1:18" ht="57.6">
       <c r="A2" s="5" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>139</v>
@@ -13840,11 +13685,11 @@
         <v>64</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="9" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="G2" s="8"/>
       <c r="H2" s="7" t="s">
@@ -13879,7 +13724,7 @@
     </row>
     <row r="3" spans="1:18" ht="57.6">
       <c r="A3" s="5" t="s">
-        <v>752</v>
+        <v>748</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>139</v>
@@ -13888,7 +13733,7 @@
         <v>64</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="5"/>
@@ -13925,7 +13770,7 @@
     </row>
     <row r="4" spans="1:18" ht="57.6">
       <c r="A4" s="5" t="s">
-        <v>750</v>
+        <v>746</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>139</v>
@@ -13934,7 +13779,7 @@
         <v>64</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="5"/>
@@ -13971,7 +13816,7 @@
     </row>
     <row r="5" spans="1:18" ht="72">
       <c r="A5" s="5" t="s">
-        <v>749</v>
+        <v>745</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>139</v>
@@ -13980,11 +13825,11 @@
         <v>64</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="5" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="G5" s="8"/>
       <c r="H5" s="7" t="s">
@@ -14029,7 +13874,7 @@
         <v>64</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="9"/>
@@ -14067,7 +13912,7 @@
     </row>
     <row r="7" spans="1:18" ht="43.2">
       <c r="A7" s="5" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>139</v>
@@ -14076,11 +13921,11 @@
         <v>64</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="5" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="G7" s="8"/>
       <c r="H7" s="7" t="s">
@@ -14216,7 +14061,7 @@
         <v>62</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -14227,7 +14072,7 @@
         <v>64</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="J2" s="8"/>
       <c r="K2" s="3"/>
@@ -14258,7 +14103,7 @@
         <v>64</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="J3" s="8"/>
       <c r="K3" s="3"/>
@@ -14277,7 +14122,7 @@
         <v>62</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -14288,7 +14133,7 @@
         <v>64</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="J4" s="8"/>
       <c r="K4" s="3"/>
@@ -14298,7 +14143,7 @@
     </row>
     <row r="5" spans="1:19" ht="43.2">
       <c r="A5" s="5" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>139</v>
@@ -14307,11 +14152,11 @@
         <v>62</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="7" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>103</v>
@@ -14320,7 +14165,7 @@
         <v>61</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="J5" s="8"/>
       <c r="K5" s="3" t="s">
@@ -14347,7 +14192,7 @@
     </row>
     <row r="6" spans="1:19" ht="28.8">
       <c r="A6" s="5" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>139</v>
@@ -14356,7 +14201,7 @@
         <v>62</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
@@ -14401,7 +14246,7 @@
         <v>62</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
@@ -14444,7 +14289,7 @@
         <v>61</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="J8" s="8"/>
       <c r="K8" s="3"/>
@@ -14474,7 +14319,7 @@
         <v>64</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="J9" s="8"/>
       <c r="K9" s="3"/>
@@ -14493,7 +14338,7 @@
         <v>62</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
@@ -14504,7 +14349,7 @@
         <v>64</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="28.8">
@@ -14518,7 +14363,7 @@
         <v>62</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
@@ -14529,7 +14374,7 @@
         <v>59</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
       <c r="J11" s="8"/>
       <c r="K11" s="3"/>
@@ -14645,7 +14490,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="C11" t="s">
-        <v>936</v>
+        <v>930</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -14693,7 +14538,7 @@
         <v>121</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>967</v>
+        <v>949</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>122</v>
@@ -14728,13 +14573,13 @@
         <v>113</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>124</v>
@@ -14746,20 +14591,20 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>971</v>
+        <v>953</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>970</v>
+        <v>952</v>
       </c>
       <c r="D4" t="s">
         <v>125</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3" t="s">
-        <v>969</v>
+        <v>951</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>968</v>
+        <v>950</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -14770,17 +14615,17 @@
         <v>114</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>970</v>
+        <v>952</v>
       </c>
       <c r="D5" t="s">
         <v>125</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>969</v>
+        <v>951</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>968</v>
+        <v>950</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -14788,10 +14633,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>936</v>
+        <v>930</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>937</v>
+        <v>931</v>
       </c>
       <c r="D6" t="s">
         <v>125</v>

</xml_diff>

<commit_message>
Added code for Firefox , Edge browser execution in framework - 7 April 2026
</commit_message>
<xml_diff>
--- a/SeleniumJavaFramework/TestData/TestData.xlsx
+++ b/SeleniumJavaFramework/TestData/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tales\git\SeleniumFramework\SeleniumJavaFramework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E71423-4F75-4240-A837-D40F936EC4C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F880171-C8DE-4A19-9DC7-71765EDC4B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FrenchMappings" sheetId="38" state="hidden" r:id="rId1"/>
@@ -3286,14 +3286,14 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>5869388</xdr:colOff>
-          <xdr:row>298</xdr:row>
-          <xdr:rowOff>184205</xdr:rowOff>
+          <xdr:row>295</xdr:row>
+          <xdr:rowOff>77857</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>265375</xdr:colOff>
-          <xdr:row>300</xdr:row>
-          <xdr:rowOff>95084</xdr:rowOff>
+          <xdr:row>296</xdr:row>
+          <xdr:rowOff>174266</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -9223,14 +9223,14 @@
               <from>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>299</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
+                <xdr:row>295</xdr:row>
+                <xdr:rowOff>76200</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>266700</xdr:colOff>
-                <xdr:row>300</xdr:row>
-                <xdr:rowOff>91440</xdr:rowOff>
+                <xdr:row>296</xdr:row>
+                <xdr:rowOff>175260</xdr:rowOff>
               </to>
             </anchor>
           </controlPr>
@@ -11384,7 +11384,7 @@
         <v>13</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>14</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>